<commit_message>
add checking info to exported file in actual stock taking
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportActualStockTakingTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportActualStockTakingTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cong-\OneDrive\Tài liệu\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project_Code\kvc-wh-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81779505-7352-42CE-A136-267E86DB71A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15E450F5-05F4-4847-A872-CE325DBFD5A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1710" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11235" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tồn kho" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Số PO</t>
   </si>
@@ -52,6 +52,12 @@
   </si>
   <si>
     <t>Số hộp thực tế</t>
+  </si>
+  <si>
+    <t>Tồn kho check</t>
+  </si>
+  <si>
+    <t>Số hộp check</t>
   </si>
 </sst>
 </file>
@@ -404,20 +410,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.44140625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="26.88671875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" style="5" customWidth="1"/>
-    <col min="4" max="5" width="19.109375" style="5" customWidth="1"/>
-    <col min="6" max="6" width="20.5546875" customWidth="1"/>
-    <col min="7" max="7" width="21.44140625" customWidth="1"/>
-    <col min="8" max="8" width="20.109375" customWidth="1"/>
-    <col min="9" max="9" width="36.33203125" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="26.85546875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" style="5" customWidth="1"/>
+    <col min="4" max="5" width="19.140625" style="5" customWidth="1"/>
+    <col min="6" max="7" width="20.5703125" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" customWidth="1"/>
+    <col min="9" max="10" width="20.140625" customWidth="1"/>
+    <col min="11" max="11" width="36.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -437,12 +443,18 @@
         <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add checking location code in export actual stock taking
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportActualStockTakingTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportActualStockTakingTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project_Code\kvc-wh-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15E450F5-05F4-4847-A872-CE325DBFD5A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D56FD43-7BA4-4D49-8B05-78B96230D982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11235" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tồn kho" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Số PO</t>
   </si>
@@ -58,6 +58,9 @@
   </si>
   <si>
     <t>Số hộp check</t>
+  </si>
+  <si>
+    <t>BIN# Check</t>
   </si>
 </sst>
 </file>
@@ -410,20 +413,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.42578125" style="3" customWidth="1"/>
     <col min="2" max="2" width="26.85546875" style="3" customWidth="1"/>
     <col min="3" max="3" width="20.7109375" style="5" customWidth="1"/>
-    <col min="4" max="5" width="19.140625" style="5" customWidth="1"/>
-    <col min="6" max="7" width="20.5703125" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" customWidth="1"/>
-    <col min="9" max="10" width="20.140625" customWidth="1"/>
-    <col min="11" max="11" width="36.28515625" customWidth="1"/>
+    <col min="4" max="6" width="19.140625" style="5" customWidth="1"/>
+    <col min="7" max="8" width="20.5703125" customWidth="1"/>
+    <col min="9" max="9" width="21.42578125" customWidth="1"/>
+    <col min="10" max="11" width="20.140625" customWidth="1"/>
+    <col min="12" max="12" width="36.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -437,24 +440,27 @@
         <v>5</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
order sending checking by result, add item name into export stock taking
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportActualStockTakingTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportActualStockTakingTemplate.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project_Code\kvc-wh-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project_Code\kvc-wh-be\target\classes\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D56FD43-7BA4-4D49-8B05-78B96230D982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27B61C7E-C002-4A24-94C6-C2073769B9B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tồn kho" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Số PO</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>BIN# Check</t>
+  </si>
+  <si>
+    <t>Tên NVL</t>
   </si>
 </sst>
 </file>
@@ -413,54 +416,57 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="26.85546875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" style="5" customWidth="1"/>
-    <col min="4" max="6" width="19.140625" style="5" customWidth="1"/>
-    <col min="7" max="8" width="20.5703125" customWidth="1"/>
-    <col min="9" max="9" width="21.42578125" customWidth="1"/>
-    <col min="10" max="11" width="20.140625" customWidth="1"/>
-    <col min="12" max="12" width="36.28515625" customWidth="1"/>
+    <col min="1" max="2" width="21.42578125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="26.85546875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="5" customWidth="1"/>
+    <col min="5" max="7" width="19.140625" style="5" customWidth="1"/>
+    <col min="8" max="9" width="20.5703125" customWidth="1"/>
+    <col min="10" max="10" width="21.42578125" customWidth="1"/>
+    <col min="11" max="12" width="20.140625" customWidth="1"/>
+    <col min="13" max="13" width="36.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>